<commit_message>
docs: update Sprint 3 test tracker and evidence
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-3-test-cases.xlsx
+++ b/docs/testing/sprint-3-test-cases.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb94a9f41dd5540c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R72fc655d05f44057"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="3" r:id="Re40273633a694041"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6d59e2284b414eb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R518adfbe1ff441ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="3" r:id="Reb815341ac5548f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,9 +15,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0%"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="10">
     <x:font>
@@ -134,7 +135,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="78">
+  <x:cellXfs count="84">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -329,6 +330,20 @@
     <x:xf numFmtId="201" fontId="9" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -340,7 +355,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -351,7 +366,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -362,7 +377,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -373,7 +388,7 @@
         <x:color rgb="FF374151"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5E7EB"/>
         </x:patternFill>
       </x:fill>
@@ -384,7 +399,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -532,7 +547,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4c6dcea3cf0c4e16"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb0368c68b48944cc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -780,11 +795,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
@@ -804,7 +819,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="13" t="str">
-        <x:v>Sprint 3: Application Documents and Interview Preparation | 7 Sep to 18 Sep 2026</x:v>
+        <x:v>Sprint 3: Application Documents and Interview Preparation | 7 Sep to 18 Sep 2026 | Updated 13 Sep 2026</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -848,14 +863,14 @@
       </x:c>
       <x:c r="E5" s="68" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Pass")</x:f>
-        <x:v>26</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="F5" t="str">
         <x:v>Executed/Ready</x:v>
       </x:c>
       <x:c r="G5" t="n">
         <x:f>E5+E6+E8+E9</x:f>
-        <x:v>41</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -878,7 +893,7 @@
       </x:c>
       <x:c r="G6" s="36" t="n">
         <x:f>IF(B7=0,0,E7/B7)</x:f>
-        <x:v>0.59</x:v>
+        <x:v>0.5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -895,7 +910,7 @@
       </x:c>
       <x:c r="E7" s="70" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Blocked")</x:f>
-        <x:v>59</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -904,7 +919,7 @@
       </x:c>
       <x:c r="B8" s="41" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Pass")</x:f>
-        <x:v>26</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C8" s="34"/>
       <x:c r="D8" s="34" t="str">
@@ -912,7 +927,7 @@
       </x:c>
       <x:c r="E8" s="71" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Not Run")</x:f>
-        <x:v>15</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -938,7 +953,7 @@
       </x:c>
       <x:c r="B10" s="49" t="n">
         <x:f>COUNTIF('Test Cases'!$L$6:$L$105,"Blocked")</x:f>
-        <x:v>59</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C10" s="34"/>
       <x:c r="D10" s="34"/>
@@ -976,105 +991,124 @@
       <x:c r="G13" s="34" t="str"/>
       <x:c r="H13" s="34" t="str"/>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="34" t="str">
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="82" t="str">
         <x:v>WBS 6.2 AI prompt templates &amp; safety</x:v>
       </x:c>
-      <x:c r="B14" s="34" t="str">
+      <x:c r="B14" s="83" t="str">
         <x:v>Jerald</x:v>
       </x:c>
-      <x:c r="C14" s="34" t="str">
+      <x:c r="C14" s="83" t="str">
         <x:v>Merged / verified</x:v>
       </x:c>
-      <x:c r="D14" s="34" t="str">
+      <x:c r="D14" s="83" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="E14" s="34" t="str">
+      <x:c r="E14" s="83" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="F14" s="34" t="str"/>
       <x:c r="G14" s="34" t="str"/>
       <x:c r="H14" s="34" t="str"/>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="34" t="str">
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="82" t="str">
         <x:v>WBS 6.3 Resume generation backend</x:v>
       </x:c>
-      <x:c r="B15" s="34" t="str">
+      <x:c r="B15" s="83" t="str">
         <x:v>MD</x:v>
       </x:c>
-      <x:c r="C15" s="34" t="str">
-        <x:v>Merged</x:v>
-      </x:c>
-      <x:c r="D15" s="34" t="str">
+      <x:c r="C15" s="83" t="str">
+        <x:v>Merged / verified</x:v>
+      </x:c>
+      <x:c r="D15" s="83" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="E15" s="34" t="str">
-        <x:v>Team-level integration verification still planned</x:v>
+      <x:c r="E15" s="83" t="str">
+        <x:v>Resume backend tests pass on current shared backend baseline</x:v>
       </x:c>
       <x:c r="F15" s="34" t="str"/>
       <x:c r="G15" s="34" t="str"/>
       <x:c r="H15" s="34" t="str"/>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="34" t="str">
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A16" s="82" t="str">
         <x:v>WBS 6.4 Cover letter generation backend</x:v>
       </x:c>
-      <x:c r="B16" s="34" t="str">
+      <x:c r="B16" s="83" t="str">
         <x:v>MD</x:v>
       </x:c>
-      <x:c r="C16" s="34" t="str">
-        <x:v>In progress / not integrated</x:v>
-      </x:c>
-      <x:c r="D16" s="34" t="str">
+      <x:c r="C16" s="83" t="str">
+        <x:v>Merged / verified</x:v>
+      </x:c>
+      <x:c r="D16" s="83" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="E16" s="34" t="str">
-        <x:v>Blocks WBS 6.8</x:v>
+      <x:c r="E16" s="83" t="str">
+        <x:v>48/48 documents tests passed; merged into feature/sprint-3</x:v>
       </x:c>
       <x:c r="F16" s="34" t="str"/>
       <x:c r="G16" s="34" t="str"/>
       <x:c r="H16" s="34" t="str"/>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="34" t="str">
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="82" t="str">
         <x:v>WBS 6.5 Resume and cover letter interface</x:v>
       </x:c>
-      <x:c r="B17" s="34" t="str">
+      <x:c r="B17" s="83" t="str">
         <x:v>Joyee</x:v>
       </x:c>
-      <x:c r="C17" s="34" t="str">
+      <x:c r="C17" s="83" t="str">
         <x:v>Not integrated</x:v>
       </x:c>
-      <x:c r="D17" s="34" t="str">
+      <x:c r="D17" s="83" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="E17" s="34" t="str">
+      <x:c r="E17" s="83" t="str">
         <x:v>Blocks WBS 6.8</x:v>
       </x:c>
       <x:c r="F17" s="34" t="str"/>
       <x:c r="G17" s="34" t="str"/>
       <x:c r="H17" s="34" t="str"/>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="34" t="str">
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A18" s="82" t="str">
         <x:v>WBS 6.6 Interview question and feedback API</x:v>
       </x:c>
-      <x:c r="B18" s="34" t="str">
+      <x:c r="B18" s="83" t="str">
         <x:v>Jerald</x:v>
       </x:c>
-      <x:c r="C18" s="34" t="str">
-        <x:v>PR #38 open</x:v>
-      </x:c>
-      <x:c r="D18" s="34" t="str">
+      <x:c r="C18" s="83" t="str">
+        <x:v>Merged / verified</x:v>
+      </x:c>
+      <x:c r="D18" s="83" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="E18" s="34" t="str">
-        <x:v>Merge required before WBS 6.8</x:v>
+      <x:c r="E18" s="83" t="str">
+        <x:v>38/38 focused tests passed; merged into feature/sprint-3</x:v>
       </x:c>
       <x:c r="F18" s="34" t="str"/>
       <x:c r="G18" s="34" t="str"/>
       <x:c r="H18" s="34" t="str"/>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="82" t="str">
+        <x:v>WBS 6.7 Interview preparation interface</x:v>
+      </x:c>
+      <x:c r="B19" s="83" t="str">
+        <x:v>Joyee</x:v>
+      </x:c>
+      <x:c r="C19" s="83" t="str">
+        <x:v>Not integrated</x:v>
+      </x:c>
+      <x:c r="D19" s="83" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E19" s="83" t="str">
+        <x:v>Blocks WBS 6.8</x:v>
+      </x:c>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="28" t="str">
@@ -1104,7 +1138,7 @@
       <x:c r="G21" s="34" t="str"/>
       <x:c r="H21" s="34" t="str"/>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A22" s="34" t="str">
         <x:v>6.8 integration</x:v>
       </x:c>
@@ -1112,7 +1146,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="C22" s="34" t="str">
-        <x:v>Do not start full integration until WBS 6.3, 6.4, 6.5, 6.6, and 6.7 are merged/available.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged. Full integration waits for WBS 6.5 and 6.7.</x:v>
       </x:c>
       <x:c r="D22" s="34" t="str"/>
       <x:c r="E22" s="34" t="str"/>
@@ -1120,7 +1154,7 @@
       <x:c r="G22" s="34" t="str"/>
       <x:c r="H22" s="34" t="str"/>
     </x:row>
-    <x:row r="23">
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A23" s="34" t="str">
         <x:v>6.9 Sprint 3 testing</x:v>
       </x:c>
@@ -1128,7 +1162,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="C23" s="34" t="str">
-        <x:v>Starts after WBS 6.8 integration passes.</x:v>
+        <x:v>Starts after WBS 6.8 integration passes. Interim backend checks do not close WBS 6.9.</x:v>
       </x:c>
       <x:c r="D23" s="34" t="str"/>
       <x:c r="E23" s="34" t="str"/>
@@ -1136,7 +1170,7 @@
       <x:c r="G23" s="34" t="str"/>
       <x:c r="H23" s="34" t="str"/>
     </x:row>
-    <x:row r="24">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="34" t="str">
         <x:v>Blocked != Fail</x:v>
       </x:c>
@@ -1152,7 +1186,7 @@
       <x:c r="G24" s="34" t="str"/>
       <x:c r="H24" s="34" t="str"/>
     </x:row>
-    <x:row r="25">
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A25" s="34" t="str">
         <x:v>Evidence</x:v>
       </x:c>
@@ -1176,7 +1210,7 @@
     <x:mergeCell ref="A20:H20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6440d9648055483c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3c591abda9646c7"/>
 </x:worksheet>
 </file>
 
@@ -1361,16 +1395,24 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L6" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M6" s="34" t="str"/>
-      <x:c r="N6" s="34" t="str"/>
-      <x:c r="O6" s="34" t="str"/>
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="M6" s="34" t="str">
+        <x:v>WBS 6.5; WBS 6.7</x:v>
+      </x:c>
+      <x:c r="N6" s="34" t="str">
+        <x:v>Current feature/sprint-3 backend baseline is current and clean at merge commit 7eac135. Full WBS 6.8 baseline remains blocked until WBS 6.5 and 6.7 are merged.</x:v>
+      </x:c>
+      <x:c r="O6" s="34" t="str">
+        <x:v>S3-EV-009</x:v>
+      </x:c>
       <x:c r="P6" s="34" t="str"/>
       <x:c r="Q6" s="34" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="R6" s="34" t="str"/>
+      <x:c r="R6" s="34" t="str">
+        <x:v>Interim branch verification completed. Rerun as a final WBS 6.8 entry check after frontend predecessors merge.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="34" t="str">
@@ -1407,16 +1449,22 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="L7" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M7" s="34" t="str"/>
-      <x:c r="N7" s="34" t="str"/>
-      <x:c r="O7" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M7" s="34"/>
+      <x:c r="N7" s="34" t="str">
+        <x:v>Django system check passed on current feature/sprint-3 backend baseline with no issues.</x:v>
+      </x:c>
+      <x:c r="O7" s="34" t="str">
+        <x:v>S3-EV-009</x:v>
+      </x:c>
       <x:c r="P7" s="34" t="str"/>
       <x:c r="Q7" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R7" s="34" t="str"/>
+      <x:c r="R7" s="34" t="str">
+        <x:v>Interim backend baseline pass. Rerun after WBS 6.5 and 6.7 merge before final Sprint 3 exit.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="34" t="str">
@@ -1453,16 +1501,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L8" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M8" s="34" t="str"/>
-      <x:c r="N8" s="34" t="str"/>
-      <x:c r="O8" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M8" s="34"/>
+      <x:c r="N8" s="34" t="str">
+        <x:v>makemigrations --check reported no changes. Test database migrations applied successfully during the 410-test regression run.</x:v>
+      </x:c>
+      <x:c r="O8" s="34" t="str">
+        <x:v>S3-EV-009</x:v>
+      </x:c>
       <x:c r="P8" s="34" t="str"/>
       <x:c r="Q8" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R8" s="34" t="str"/>
+      <x:c r="R8" s="34" t="str">
+        <x:v>Interim backend baseline pass. Final migration review remains part of WBS 6.9 after WBS 6.8.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="34" t="str">
@@ -2191,17 +2245,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L23" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M23" s="34" t="str"/>
-      <x:c r="N23" s="34" t="str"/>
-      <x:c r="O23" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M23" s="34"/>
+      <x:c r="N23" s="34" t="str">
+        <x:v>Authentication-required resume API test passed in the shared 410-test backend regression.</x:v>
+      </x:c>
+      <x:c r="O23" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P23" s="34" t="str"/>
       <x:c r="Q23" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R23" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2239,17 +2297,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L24" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M24" s="34" t="str"/>
-      <x:c r="N24" s="34" t="str"/>
-      <x:c r="O24" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M24" s="34"/>
+      <x:c r="N24" s="34" t="str">
+        <x:v>Unexpected client ownership/profile/prompt fields were rejected by automated resume API tests.</x:v>
+      </x:c>
+      <x:c r="O24" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P24" s="34" t="str"/>
       <x:c r="Q24" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
       <x:c r="R24" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2287,17 +2349,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L25" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M25" s="34" t="str"/>
-      <x:c r="N25" s="34" t="str"/>
-      <x:c r="O25" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M25" s="34"/>
+      <x:c r="N25" s="34" t="str">
+        <x:v>Authenticated Student profile isolation and approved profile-context tests passed.</x:v>
+      </x:c>
+      <x:c r="O25" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P25" s="34" t="str"/>
       <x:c r="Q25" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R25" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2335,17 +2401,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L26" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M26" s="34" t="str"/>
-      <x:c r="N26" s="34" t="str"/>
-      <x:c r="O26" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M26" s="34"/>
+      <x:c r="N26" s="34" t="str">
+        <x:v>Resume service used the approved RESUME_GENERATION provider/output contract in automated tests.</x:v>
+      </x:c>
+      <x:c r="O26" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P26" s="34" t="str"/>
       <x:c r="Q26" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R26" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2383,17 +2453,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L27" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M27" s="34" t="str"/>
-      <x:c r="N27" s="34" t="str"/>
-      <x:c r="O27" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M27" s="34"/>
+      <x:c r="N27" s="34" t="str">
+        <x:v>Structured ResumeDraft response and required review flags passed automated API tests.</x:v>
+      </x:c>
+      <x:c r="O27" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P27" s="34" t="str"/>
       <x:c r="Q27" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R27" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2431,17 +2505,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L28" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M28" s="34" t="str"/>
-      <x:c r="N28" s="34" t="str"/>
-      <x:c r="O28" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M28" s="34"/>
+      <x:c r="N28" s="34" t="str">
+        <x:v>Default resume provider seam failed closed with controlled 503 behaviour in automated tests.</x:v>
+      </x:c>
+      <x:c r="O28" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P28" s="34" t="str"/>
       <x:c r="Q28" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R28" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2479,17 +2557,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L29" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M29" s="34" t="str"/>
-      <x:c r="N29" s="34" t="str"/>
-      <x:c r="O29" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M29" s="34"/>
+      <x:c r="N29" s="34" t="str">
+        <x:v>AIProviderTimeoutError propagation and controlled shared AI service failure handling passed automated documents tests.</x:v>
+      </x:c>
+      <x:c r="O29" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P29" s="34" t="str"/>
       <x:c r="Q29" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R29" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2527,17 +2609,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L30" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M30" s="34" t="str"/>
-      <x:c r="N30" s="34" t="str"/>
-      <x:c r="O30" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M30" s="34"/>
+      <x:c r="N30" s="34" t="str">
+        <x:v>Private profile fields were excluded from the resume provider prompt in automated privacy tests.</x:v>
+      </x:c>
+      <x:c r="O30" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P30" s="34" t="str"/>
       <x:c r="Q30" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
       <x:c r="R30" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2575,17 +2661,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L31" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M31" s="34" t="str"/>
-      <x:c r="N31" s="34" t="str"/>
-      <x:c r="O31" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M31" s="34"/>
+      <x:c r="N31" s="34" t="str">
+        <x:v>All resume-generation automated tests included in the current shared backend regression passed.</x:v>
+      </x:c>
+      <x:c r="O31" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P31" s="34" t="str"/>
       <x:c r="Q31" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R31" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2623,17 +2713,21 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L32" s="34" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M32" s="34" t="str"/>
-      <x:c r="N32" s="34" t="str"/>
-      <x:c r="O32" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M32" s="34"/>
+      <x:c r="N32" s="34" t="str">
+        <x:v>Current feature/sprint-3 full backend regression passed 410/410 tests.</x:v>
+      </x:c>
+      <x:c r="O32" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P32" s="34" t="str"/>
       <x:c r="Q32" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R32" s="34" t="str">
-        <x:v>WBS 6.3 is merged. Execute at Sprint 3 team-integration checkpoint and attach evidence.</x:v>
+        <x:v>Verified on the current merged feature/sprint-3 backend baseline. Dedicated WBS 6.3 evidence remains useful for team closeout.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2671,18 +2765,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L33" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M33" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N33" s="34" t="str"/>
-      <x:c r="O33" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M33" s="34"/>
+      <x:c r="N33" s="34" t="str">
+        <x:v>Cover-letter authentication-required test passed.</x:v>
+      </x:c>
+      <x:c r="O33" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P33" s="34" t="str"/>
       <x:c r="Q33" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R33" s="34" t="str"/>
+      <x:c r="R33" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="34" t="str">
@@ -2719,18 +2817,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L34" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M34" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N34" s="34" t="str"/>
-      <x:c r="O34" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M34" s="34"/>
+      <x:c r="N34" s="34" t="str">
+        <x:v>Validated job-description request contract passed automated tests.</x:v>
+      </x:c>
+      <x:c r="O34" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P34" s="34" t="str"/>
       <x:c r="Q34" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R34" s="34" t="str"/>
+      <x:c r="R34" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="34" t="str">
@@ -2767,18 +2869,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L35" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M35" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N35" s="34" t="str"/>
-      <x:c r="O35" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M35" s="34"/>
+      <x:c r="N35" s="34" t="str">
+        <x:v>Blank job description was rejected by API and input-contract tests.</x:v>
+      </x:c>
+      <x:c r="O35" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P35" s="34" t="str"/>
       <x:c r="Q35" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R35" s="34" t="str"/>
+      <x:c r="R35" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="34" t="str">
@@ -2815,18 +2921,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L36" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M36" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N36" s="34" t="str"/>
-      <x:c r="O36" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M36" s="34"/>
+      <x:c r="N36" s="34" t="str">
+        <x:v>Client ownership identifiers, prompt overrides, and unexpected fields were rejected.</x:v>
+      </x:c>
+      <x:c r="O36" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P36" s="34" t="str"/>
       <x:c r="Q36" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R36" s="34" t="str"/>
+      <x:c r="R36" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="34" t="str">
@@ -2863,18 +2973,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L37" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M37" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N37" s="34" t="str"/>
-      <x:c r="O37" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M37" s="34"/>
+      <x:c r="N37" s="34" t="str">
+        <x:v>Authenticated Student profile supplied approved cover-letter context and cross-user selection was blocked.</x:v>
+      </x:c>
+      <x:c r="O37" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P37" s="34" t="str"/>
       <x:c r="Q37" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R37" s="34" t="str"/>
+      <x:c r="R37" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="34" t="str">
@@ -2911,18 +3025,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L38" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M38" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N38" s="34" t="str"/>
-      <x:c r="O38" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M38" s="34"/>
+      <x:c r="N38" s="34" t="str">
+        <x:v>Job description remained untrusted content and instruction-like text did not become trusted instructions.</x:v>
+      </x:c>
+      <x:c r="O38" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P38" s="34" t="str"/>
       <x:c r="Q38" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R38" s="34" t="str"/>
+      <x:c r="R38" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="34" t="str">
@@ -2959,18 +3077,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L39" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M39" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N39" s="34" t="str"/>
-      <x:c r="O39" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M39" s="34"/>
+      <x:c r="N39" s="34" t="str">
+        <x:v>CoverLetterDraft contract, privacy mapping, supplied-fact boundaries, and structured output validation passed.</x:v>
+      </x:c>
+      <x:c r="O39" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P39" s="34" t="str"/>
       <x:c r="Q39" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R39" s="34" t="str"/>
+      <x:c r="R39" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="34" t="str">
@@ -3007,18 +3129,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L40" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M40" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N40" s="34" t="str"/>
-      <x:c r="O40" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M40" s="34"/>
+      <x:c r="N40" s="34" t="str">
+        <x:v>Generated cover-letter draft retained draft/requires_user_review flags.</x:v>
+      </x:c>
+      <x:c r="O40" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P40" s="34" t="str"/>
       <x:c r="Q40" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R40" s="34" t="str"/>
+      <x:c r="R40" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="34" t="str">
@@ -3055,18 +3181,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L41" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M41" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N41" s="34" t="str"/>
-      <x:c r="O41" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M41" s="34"/>
+      <x:c r="N41" s="34" t="str">
+        <x:v>Default provider seam and shared AI service failure paths returned controlled service errors.</x:v>
+      </x:c>
+      <x:c r="O41" s="34" t="str">
+        <x:v>S3-EV-004A</x:v>
+      </x:c>
       <x:c r="P41" s="34" t="str"/>
       <x:c r="Q41" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R41" s="34" t="str"/>
+      <x:c r="R41" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="34" t="str">
@@ -3103,18 +3233,22 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L42" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M42" s="34" t="str">
-        <x:v>WBS 6.4 implementation/merge</x:v>
-      </x:c>
-      <x:c r="N42" s="34" t="str"/>
-      <x:c r="O42" s="34" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M42" s="34"/>
+      <x:c r="N42" s="34" t="str">
+        <x:v>48/48 documents tests passed on the merged Sprint 3 baseline; current shared feature/sprint-3 backend regression passed 410/410.</x:v>
+      </x:c>
+      <x:c r="O42" s="34" t="str">
+        <x:v>S3-EV-004A; S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P42" s="34" t="str"/>
       <x:c r="Q42" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R42" s="34" t="str"/>
+      <x:c r="R42" s="34" t="str">
+        <x:v>WBS 6.4 is merged into feature/sprint-3 and verified against the updated Sprint 3 backend baseline.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="34" t="str">
@@ -3619,7 +3753,7 @@
         <x:v>Interview question endpoint requires JWT</x:v>
       </x:c>
       <x:c r="H53" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I53" s="34" t="str">
         <x:v>POST questions endpoint without token.</x:v>
@@ -3638,14 +3772,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O53" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P53" s="34" t="str"/>
       <x:c r="Q53" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R53" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3671,7 +3805,7 @@
         <x:v>Interview feedback endpoint requires JWT</x:v>
       </x:c>
       <x:c r="H54" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I54" s="34" t="str">
         <x:v>POST feedback endpoint without token.</x:v>
@@ -3690,14 +3824,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O54" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P54" s="34" t="str"/>
       <x:c r="Q54" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R54" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -3723,7 +3857,7 @@
         <x:v>Invalid JWT is rejected by both interview endpoints</x:v>
       </x:c>
       <x:c r="H55" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I55" s="34" t="str">
         <x:v>Use invalid bearer token.</x:v>
@@ -3742,14 +3876,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O55" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P55" s="34" t="str"/>
       <x:c r="Q55" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R55" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -3775,7 +3909,7 @@
         <x:v>Interview question request applies default count 5</x:v>
       </x:c>
       <x:c r="H56" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I56" s="34" t="str">
         <x:v>Validate request without question_count.</x:v>
@@ -3794,14 +3928,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O56" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P56" s="34" t="str"/>
       <x:c r="Q56" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R56" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -3827,7 +3961,7 @@
         <x:v>Interview question count enforces 1 to 10</x:v>
       </x:c>
       <x:c r="H57" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I57" s="34" t="str">
         <x:v>Validate 0 and 11 counts.</x:v>
@@ -3846,14 +3980,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O57" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P57" s="34" t="str"/>
       <x:c r="Q57" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R57" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -3879,7 +4013,7 @@
         <x:v>Interview question count rejects string coercion</x:v>
       </x:c>
       <x:c r="H58" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I58" s="34" t="str">
         <x:v>Submit question_count as string '5'.</x:v>
@@ -3898,14 +4032,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O58" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P58" s="34" t="str"/>
       <x:c r="Q58" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R58" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -3931,7 +4065,7 @@
         <x:v>Interview endpoints reject unexpected ownership/prompt fields</x:v>
       </x:c>
       <x:c r="H59" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I59" s="34" t="str">
         <x:v>Submit user_id, student_profile_id, or prompt fields.</x:v>
@@ -3950,14 +4084,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O59" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P59" s="34" t="str"/>
       <x:c r="Q59" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
       <x:c r="R59" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -3983,7 +4117,7 @@
         <x:v>Target role and job description remain untrusted</x:v>
       </x:c>
       <x:c r="H60" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I60" s="34" t="str">
         <x:v>Generate questions with role/job text.</x:v>
@@ -4002,14 +4136,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O60" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P60" s="34" t="str"/>
       <x:c r="Q60" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
       <x:c r="R60" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -4035,7 +4169,7 @@
         <x:v>Question generation uses approved WBS 6.2 operation/output contract</x:v>
       </x:c>
       <x:c r="H61" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I61" s="34" t="str">
         <x:v>Invoke service with fake provider.</x:v>
@@ -4054,14 +4188,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O61" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P61" s="34" t="str"/>
       <x:c r="Q61" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R61" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -4087,7 +4221,7 @@
         <x:v>Interview feedback text remains untrusted</x:v>
       </x:c>
       <x:c r="H62" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I62" s="34" t="str">
         <x:v>Generate feedback with role/question/answer.</x:v>
@@ -4106,14 +4240,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O62" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P62" s="34" t="str"/>
       <x:c r="Q62" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
       <x:c r="R62" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -4139,7 +4273,7 @@
         <x:v>Feedback generation uses approved operation/output contract</x:v>
       </x:c>
       <x:c r="H63" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I63" s="34" t="str">
         <x:v>Invoke service with fake provider.</x:v>
@@ -4158,14 +4292,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O63" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P63" s="34" t="str"/>
       <x:c r="Q63" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R63" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -4191,7 +4325,7 @@
         <x:v>Interview responses exclude hiring probability and pass/fail</x:v>
       </x:c>
       <x:c r="H64" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I64" s="34" t="str">
         <x:v>Inspect structured API responses.</x:v>
@@ -4210,14 +4344,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O64" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P64" s="34" t="str"/>
       <x:c r="Q64" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
       <x:c r="R64" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -4243,7 +4377,7 @@
         <x:v>Provider unavailable or timeout returns controlled 503</x:v>
       </x:c>
       <x:c r="H65" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I65" s="34" t="str">
         <x:v>Exercise default seam and timeout provider.</x:v>
@@ -4262,14 +4396,14 @@
         <x:v>Verified by WBS 6.6 automated tests.</x:v>
       </x:c>
       <x:c r="O65" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B</x:v>
+        <x:v>S3-EV-002F</x:v>
       </x:c>
       <x:c r="P65" s="34" t="str"/>
       <x:c r="Q65" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R65" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -4295,13 +4429,13 @@
         <x:v>Focused WBS 6.6 tests and full backend regression pass</x:v>
       </x:c>
       <x:c r="H66" s="34" t="str">
-        <x:v>WBS 6.6 implementation complete on PR #38 branch.</x:v>
+        <x:v>WBS 6.6 merged into feature/sprint-3.</x:v>
       </x:c>
       <x:c r="I66" s="34" t="str">
         <x:v>Run interviews suite, then full backend suite.</x:v>
       </x:c>
       <x:c r="J66" s="34" t="str">
-        <x:v>38/38 focused tests and 343/343 backend tests pass.</x:v>
+        <x:v>38/38 focused interview tests pass and the current full backend regression remains green.</x:v>
       </x:c>
       <x:c r="K66" s="34" t="str">
         <x:v>Jerald</x:v>
@@ -4311,17 +4445,17 @@
       </x:c>
       <x:c r="M66" s="34" t="str"/>
       <x:c r="N66" s="34" t="str">
-        <x:v>38/38 focused tests and 343/343 backend tests passed; Django check passed.</x:v>
+        <x:v>38/38 interview tests passed post-merge; current shared feature/sprint-3 full backend regression passed 410/410.</x:v>
       </x:c>
       <x:c r="O66" s="34" t="str">
-        <x:v>S3-EV-002A; S3-EV-002B; S3-EV-002C; S3-EV-002D; S3-EV-002E</x:v>
+        <x:v>S3-EV-002F; S3-EV-009A; S3-EV-009B</x:v>
       </x:c>
       <x:c r="P66" s="34" t="str"/>
       <x:c r="Q66" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
       <x:c r="R66" s="34" t="str">
-        <x:v>Component-level result. WBS 6.8 end-to-end integration remains blocked until all Sprint 3 predecessors are ready.</x:v>
+        <x:v>Component-level result verified after merge. WBS 6.8 end-to-end integration remains blocked until WBS 6.5 and 6.7 are ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -4362,7 +4496,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M67" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N67" s="34" t="str"/>
       <x:c r="O67" s="34" t="str"/>
@@ -4410,7 +4544,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M68" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N68" s="34" t="str"/>
       <x:c r="O68" s="34" t="str"/>
@@ -4458,7 +4592,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M69" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N69" s="34" t="str"/>
       <x:c r="O69" s="34" t="str"/>
@@ -4506,7 +4640,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M70" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N70" s="34" t="str"/>
       <x:c r="O70" s="34" t="str"/>
@@ -4554,7 +4688,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M71" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N71" s="34" t="str"/>
       <x:c r="O71" s="34" t="str"/>
@@ -4602,7 +4736,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M72" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N72" s="34" t="str"/>
       <x:c r="O72" s="34" t="str"/>
@@ -4650,7 +4784,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M73" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N73" s="34" t="str"/>
       <x:c r="O73" s="34" t="str"/>
@@ -4698,7 +4832,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M74" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N74" s="34" t="str"/>
       <x:c r="O74" s="34" t="str"/>
@@ -4746,7 +4880,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M75" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N75" s="34" t="str"/>
       <x:c r="O75" s="34" t="str"/>
@@ -4794,7 +4928,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M76" s="34" t="str">
-        <x:v>WBS 6.5; WBS 6.7 implementation/merge; WBS 6.6 merge</x:v>
+        <x:v>WBS 6.5; WBS 6.7 implementation/merge</x:v>
       </x:c>
       <x:c r="N76" s="34" t="str"/>
       <x:c r="O76" s="34" t="str"/>
@@ -4827,7 +4961,7 @@
         <x:v>Integrated branch contains WBS 6.3 to 6.7 deliverables</x:v>
       </x:c>
       <x:c r="H77" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I77" s="34" t="str">
         <x:v>Review feature/sprint-3 history and paths.</x:v>
@@ -4842,7 +4976,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M77" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N77" s="34" t="str"/>
       <x:c r="O77" s="34" t="str"/>
@@ -4875,7 +5009,7 @@
         <x:v>Resume UI to API flow works end to end</x:v>
       </x:c>
       <x:c r="H78" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I78" s="34" t="str">
         <x:v>Login; open Resume Builder; generate; review/edit.</x:v>
@@ -4890,7 +5024,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M78" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N78" s="34" t="str"/>
       <x:c r="O78" s="34" t="str"/>
@@ -4923,7 +5057,7 @@
         <x:v>Cover letter UI to API flow works end to end</x:v>
       </x:c>
       <x:c r="H79" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I79" s="34" t="str">
         <x:v>Login; provide one job description; generate; review/edit.</x:v>
@@ -4938,7 +5072,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M79" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N79" s="34" t="str"/>
       <x:c r="O79" s="34" t="str"/>
@@ -4971,7 +5105,7 @@
         <x:v>Interview question UI to API flow works end to end</x:v>
       </x:c>
       <x:c r="H80" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I80" s="34" t="str">
         <x:v>Login; open interview prep; generate questions.</x:v>
@@ -4986,7 +5120,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M80" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N80" s="34" t="str"/>
       <x:c r="O80" s="34" t="str"/>
@@ -5019,7 +5153,7 @@
         <x:v>Interview feedback UI to API flow works end to end</x:v>
       </x:c>
       <x:c r="H81" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I81" s="34" t="str">
         <x:v>Answer generated question and request feedback.</x:v>
@@ -5034,7 +5168,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M81" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N81" s="34" t="str"/>
       <x:c r="O81" s="34" t="str"/>
@@ -5067,7 +5201,7 @@
         <x:v>Document and interview flows preserve authenticated Student context</x:v>
       </x:c>
       <x:c r="H82" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I82" s="34" t="str">
         <x:v>Run flows with Student A and Student B.</x:v>
@@ -5082,7 +5216,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M82" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N82" s="34" t="str"/>
       <x:c r="O82" s="34" t="str"/>
@@ -5115,7 +5249,7 @@
         <x:v>Resume flow rejects client profile/prompt manipulation</x:v>
       </x:c>
       <x:c r="H83" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I83" s="34" t="str">
         <x:v>Attempt UI/API manipulation with ownership/prompt fields.</x:v>
@@ -5130,7 +5264,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M83" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N83" s="34" t="str"/>
       <x:c r="O83" s="34" t="str"/>
@@ -5163,7 +5297,7 @@
         <x:v>Cover letter flow rejects prompt injection as instruction</x:v>
       </x:c>
       <x:c r="H84" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I84" s="34" t="str">
         <x:v>Use instruction-like text inside job description.</x:v>
@@ -5178,7 +5312,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M84" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N84" s="34" t="str"/>
       <x:c r="O84" s="34" t="str"/>
@@ -5211,7 +5345,7 @@
         <x:v>Interview flow rejects prompt injection as instruction</x:v>
       </x:c>
       <x:c r="H85" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I85" s="34" t="str">
         <x:v>Use instruction-like role/job/answer text.</x:v>
@@ -5226,7 +5360,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M85" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N85" s="34" t="str"/>
       <x:c r="O85" s="34" t="str"/>
@@ -5259,7 +5393,7 @@
         <x:v>Generated content consistently shows review-required state</x:v>
       </x:c>
       <x:c r="H86" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I86" s="34" t="str">
         <x:v>Generate resume, cover letter, interview content.</x:v>
@@ -5274,7 +5408,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M86" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N86" s="34" t="str"/>
       <x:c r="O86" s="34" t="str"/>
@@ -5307,7 +5441,7 @@
         <x:v>Provider unavailable state is consistent across Sprint 3 features</x:v>
       </x:c>
       <x:c r="H87" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I87" s="34" t="str">
         <x:v>Trigger default/unavailable provider across features.</x:v>
@@ -5322,7 +5456,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M87" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N87" s="34" t="str"/>
       <x:c r="O87" s="34" t="str"/>
@@ -5355,7 +5489,7 @@
         <x:v>Invalid/expired authentication is handled consistently</x:v>
       </x:c>
       <x:c r="H88" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I88" s="34" t="str">
         <x:v>Run document/interview requests with invalid or expired token.</x:v>
@@ -5370,7 +5504,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M88" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N88" s="34" t="str"/>
       <x:c r="O88" s="34" t="str"/>
@@ -5403,7 +5537,7 @@
         <x:v>Navigation preserves intended document/interview context</x:v>
       </x:c>
       <x:c r="H89" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I89" s="34" t="str">
         <x:v>Navigate between Sprint 3 pages during normal flow.</x:v>
@@ -5418,7 +5552,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M89" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N89" s="34" t="str"/>
       <x:c r="O89" s="34" t="str"/>
@@ -5451,7 +5585,7 @@
         <x:v>Full Sprint 3 happy-path journey completes without blocking defect</x:v>
       </x:c>
       <x:c r="H90" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, and 6.7 merged into feature/sprint-3.</x:v>
+        <x:v>WBS 6.3, 6.4, and 6.6 are merged into feature/sprint-3. WBS 6.5 and 6.7 must be merged before full WBS 6.8 integration.</x:v>
       </x:c>
       <x:c r="I90" s="34" t="str">
         <x:v>Login -&gt; profile -&gt; resume -&gt; cover letter -&gt; interview questions -&gt; feedback.</x:v>
@@ -5466,7 +5600,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M90" s="34" t="str">
-        <x:v>WBS 6.3, 6.4, 6.5, 6.6, 6.7</x:v>
+        <x:v>WBS 6.5; WBS 6.7</x:v>
       </x:c>
       <x:c r="N90" s="34" t="str"/>
       <x:c r="O90" s="34" t="str"/>
@@ -5516,13 +5650,19 @@
       <x:c r="M91" s="34" t="str">
         <x:v>WBS 6.8</x:v>
       </x:c>
-      <x:c r="N91" s="34" t="str"/>
-      <x:c r="O91" s="34" t="str"/>
+      <x:c r="N91" s="34" t="str">
+        <x:v>Interim pre-WBS 6.8 shared backend baseline passed 410/410 tests on feature/sprint-3.</x:v>
+      </x:c>
+      <x:c r="O91" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
       <x:c r="P91" s="34" t="str"/>
       <x:c r="Q91" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R91" s="34" t="str"/>
+      <x:c r="R91" s="34" t="str">
+        <x:v>Status remains Blocked because the final WBS 6.9 regression must run after WBS 6.8 integration.</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="34" t="str">
@@ -5564,13 +5704,19 @@
       <x:c r="M92" s="34" t="str">
         <x:v>WBS 6.8</x:v>
       </x:c>
-      <x:c r="N92" s="34" t="str"/>
-      <x:c r="O92" s="34" t="str"/>
+      <x:c r="N92" s="34" t="str">
+        <x:v>Interim Django system check passed with no issues on feature/sprint-3.</x:v>
+      </x:c>
+      <x:c r="O92" s="34" t="str">
+        <x:v>S3-EV-009B</x:v>
+      </x:c>
       <x:c r="P92" s="34" t="str"/>
       <x:c r="Q92" s="34" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R92" s="34" t="str"/>
+      <x:c r="R92" s="34" t="str">
+        <x:v>Status remains Blocked because this check must be rerun after WBS 6.8 integration.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="34" t="str">
@@ -5612,13 +5758,19 @@
       <x:c r="M93" s="34" t="str">
         <x:v>WBS 6.8</x:v>
       </x:c>
-      <x:c r="N93" s="34" t="str"/>
-      <x:c r="O93" s="34" t="str"/>
+      <x:c r="N93" s="34" t="str">
+        <x:v>Interim makemigrations --check reported no changes on feature/sprint-3.</x:v>
+      </x:c>
+      <x:c r="O93" s="34" t="str">
+        <x:v>S3-EV-009B</x:v>
+      </x:c>
       <x:c r="P93" s="34" t="str"/>
       <x:c r="Q93" s="34" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R93" s="34" t="str"/>
+      <x:c r="R93" s="34" t="str">
+        <x:v>Status remains Blocked because final migration verification belongs to post-WBS 6.8 Sprint 3 testing.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="34" t="str">
@@ -6235,7 +6387,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re48a7e05d54e4c1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74920cca6980474d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6493,7 +6645,7 @@
       </x:c>
       <x:c r="I11" s="34" t="str"/>
       <x:c r="J11" s="34" t="str">
-        <x:v>PR #38 branch evidence</x:v>
+        <x:v>WBS 6.6 component evidence captured before merge; PR #38 is now merged into feature/sprint-3.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -6523,7 +6675,7 @@
       </x:c>
       <x:c r="I12" s="34" t="str"/>
       <x:c r="J12" s="34" t="str">
-        <x:v>PR #38 branch evidence</x:v>
+        <x:v>WBS 6.6 component evidence captured before merge; PR #38 is now merged into feature/sprint-3.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -6553,7 +6705,7 @@
       </x:c>
       <x:c r="I13" s="34" t="str"/>
       <x:c r="J13" s="34" t="str">
-        <x:v>PR #38 branch evidence</x:v>
+        <x:v>WBS 6.6 component evidence captured before merge; latest shared regression is recorded in S3-EV-009.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -6583,7 +6735,7 @@
       </x:c>
       <x:c r="I14" s="34" t="str"/>
       <x:c r="J14" s="34" t="str">
-        <x:v>PR #38 branch evidence</x:v>
+        <x:v>WBS 6.6 component evidence captured before merge; latest shared regression is recorded in S3-EV-009.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -6613,7 +6765,7 @@
       </x:c>
       <x:c r="I15" s="34" t="str"/>
       <x:c r="J15" s="34" t="str">
-        <x:v>PR #38 branch evidence</x:v>
+        <x:v>WBS 6.6 branch evidence captured; PR #38 is now merged into feature/sprint-3.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -6621,59 +6773,63 @@
         <x:v>S3-EV-003</x:v>
       </x:c>
       <x:c r="B16" s="34" t="str">
-        <x:v>TBD</x:v>
+        <x:v>S3-TC-018:S3-TC-027</x:v>
       </x:c>
       <x:c r="C16" s="34" t="str">
         <x:v>6.3</x:v>
       </x:c>
       <x:c r="D16" s="34" t="str">
-        <x:v>Test Output</x:v>
+        <x:v>Screenshot</x:v>
       </x:c>
       <x:c r="E16" s="34" t="str">
-        <x:v>WBS 6.3 resume backend focused test evidence</x:v>
+        <x:v>Resume backend verification within current shared Sprint 3 backend regression</x:v>
       </x:c>
       <x:c r="F16" s="34" t="str">
-        <x:v>docs/testing/evidence/sprint-3/S3-EV-003-*</x:v>
+        <x:v>docs/testing/evidence/sprint-3/S3-EV-009A-shared-backend-regression.png</x:v>
       </x:c>
       <x:c r="G16" s="34" t="str">
         <x:v>MD</x:v>
       </x:c>
       <x:c r="H16" s="34" t="str">
-        <x:v>Planned</x:v>
-      </x:c>
-      <x:c r="I16" s="34" t="str"/>
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I16" s="79" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J16" s="34" t="str">
-        <x:v>Capture during team integration verification</x:v>
+        <x:v>Resume-generation tests are included in the verified 410-test shared backend run. Dedicated focused WBS 6.3 evidence can still be added.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="34" t="str">
-        <x:v>S3-EV-004</x:v>
+        <x:v>S3-EV-004A</x:v>
       </x:c>
       <x:c r="B17" s="34" t="str">
-        <x:v>TBD</x:v>
+        <x:v>S3-TC-028:S3-TC-037</x:v>
       </x:c>
       <x:c r="C17" s="34" t="str">
         <x:v>6.4</x:v>
       </x:c>
       <x:c r="D17" s="34" t="str">
-        <x:v>Test Output</x:v>
+        <x:v>Screenshot</x:v>
       </x:c>
       <x:c r="E17" s="34" t="str">
-        <x:v>WBS 6.4 cover-letter backend evidence</x:v>
+        <x:v>WBS 6.4 documents focused test suite</x:v>
       </x:c>
       <x:c r="F17" s="34" t="str">
-        <x:v>docs/testing/evidence/sprint-3/S3-EV-004-*</x:v>
+        <x:v>docs/testing/evidence/sprint-3/S3-EV-004A-wbs-6.4-documents-tests.png</x:v>
       </x:c>
       <x:c r="G17" s="34" t="str">
-        <x:v>MD</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="H17" s="34" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I17" s="34" t="str"/>
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I17" s="79" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J17" s="34" t="str">
-        <x:v>Blocked until WBS 6.4 ready</x:v>
+        <x:v>Fresh post-merge evidence: 48/48 documents tests passed in 31.948s; exit code 0.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -6701,7 +6857,7 @@
       <x:c r="H18" s="34" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="I18" s="34" t="str"/>
+      <x:c r="I18" s="79" t="str"/>
       <x:c r="J18" s="34" t="str">
         <x:v>Blocked until WBS 6.5 ready</x:v>
       </x:c>
@@ -6731,7 +6887,7 @@
       <x:c r="H19" s="34" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="I19" s="34" t="str"/>
+      <x:c r="I19" s="79" t="str"/>
       <x:c r="J19" s="34" t="str">
         <x:v>Blocked until WBS 6.7 ready</x:v>
       </x:c>
@@ -6761,7 +6917,7 @@
       <x:c r="H20" s="34" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="I20" s="34" t="str"/>
+      <x:c r="I20" s="79" t="str"/>
       <x:c r="J20" s="34" t="str">
         <x:v>Blocked until 6.3-6.7 ready</x:v>
       </x:c>
@@ -6791,9 +6947,105 @@
       <x:c r="H21" s="34" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="I21" s="34" t="str"/>
+      <x:c r="I21" s="79" t="str"/>
       <x:c r="J21" s="34" t="str">
         <x:v>Blocked until WBS 6.8 passes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="34" t="str">
+        <x:v>S3-EV-009A</x:v>
+      </x:c>
+      <x:c r="B22" s="34" t="str">
+        <x:v>S3-TC-001:S3-TC-003; S3-TC-018:S3-TC-027; S3-TC-037; S3-TC-061; S3-TC-086</x:v>
+      </x:c>
+      <x:c r="C22" s="34" t="str">
+        <x:v>6.3/6.4/6.6/6.8/6.9</x:v>
+      </x:c>
+      <x:c r="D22" s="34" t="str">
+        <x:v>Screenshot</x:v>
+      </x:c>
+      <x:c r="E22" s="34" t="str">
+        <x:v>Shared feature/sprint-3 full backend regression</x:v>
+      </x:c>
+      <x:c r="F22" s="34" t="str">
+        <x:v>docs/testing/evidence/sprint-3/S3-EV-009A-shared-backend-regression.png</x:v>
+      </x:c>
+      <x:c r="G22" s="34" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H22" s="34" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I22" s="79" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="J22" s="34" t="str">
+        <x:v>Fresh shared-branch evidence: 410/410 backend tests passed in 172.904s; exit code 0.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>S3-EV-009B</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>S3-TC-087:S3-TC-088</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>6.9</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Screenshot</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>Shared feature/sprint-3 Django, migration, and Git baseline checks</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>docs/testing/evidence/sprint-3/S3-EV-009B-shared-backend-checks-and-status.png</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I23" s="80" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>Django system check passed; makemigrations --check reported no changes; feature/sprint-3 was up to date and working tree clean.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>S3-EV-002F</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>S3-TC-048:S3-TC-061</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>6.6</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>Screenshot</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>WBS 6.6 post-merge focused interview test suite</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>docs/testing/evidence/sprint-3/S3-EV-002F-wbs-6.6-post-merge-interview-tests.png</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I24" s="80" t="n">
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>Fresh post-merge evidence: 38/38 interview tests passed in 9.057s; exit code 0.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6808,7 +7060,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cdd7bdf21fa42de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd7fbd3a6aeb49f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>